<commit_message>
filtered out low read samples in analyses
</commit_message>
<xml_diff>
--- a/1-data/HS-sample-info.xlsx
+++ b/1-data/HS-sample-info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bfu/Dropbox (Personal)/Papers/Multiplexed 16S/Github/CUPID-seq-protocol/1-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F084C135-9CDA-8546-A7A0-7F74B8D5370F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4230494D-FF27-FE45-A1C3-3B6144B7D343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2600" yWindow="2700" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{A6D5D2C5-6DB2-4D41-852E-3B59AF8BF0D4}"/>
   </bookViews>
@@ -2454,7 +2454,7 @@
     <t>Drug_no</t>
   </si>
   <si>
-    <t>CUPID-Seq</t>
+    <t>CUPID-seq</t>
   </si>
 </sst>
 </file>
@@ -23397,7 +23397,7 @@
   <cols>
     <col min="1" max="1" width="61.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.33203125" bestFit="1" customWidth="1"/>

</xml_diff>